<commit_message>
cluster simulation for 3 uavs
</commit_message>
<xml_diff>
--- a/results/cluster_ga/UAVs3_GRID13/revenue/UAVs3_GRID13_cluster_ga.xlsx
+++ b/results/cluster_ga/UAVs3_GRID13/revenue/UAVs3_GRID13_cluster_ga.xlsx
@@ -547,16 +547,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4751752919983119</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.64103204269862</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.32770884558207</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18.19581888939037</v>
+        <v>97.84393658296904</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.07480154907168</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.85769181230305</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.98074714773984</v>
       </c>
     </row>
   </sheetData>
@@ -605,16 +605,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5039172079996206</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.97973729979146</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.41068130381903</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.75205368823216</v>
+        <v>107.2974282079958</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.70044831758297</v>
+      </c>
+      <c r="D2" t="n">
+        <v>47.90030503421773</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.08926520926519</v>
       </c>
     </row>
   </sheetData>
@@ -663,16 +663,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5138528330135159</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.82169145101596</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.0339198253313</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.95240758627691</v>
+        <v>98.6832752499613</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.86964845735788</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.21136823109548</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.49399050872763</v>
       </c>
     </row>
   </sheetData>
@@ -721,16 +721,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4669349170289934</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.95781178522795</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.6010832853465</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.54191019484806</v>
+        <v>96.34697104099905</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.3986638553951</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.89905521318673</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.72796141062422</v>
       </c>
     </row>
   </sheetData>
@@ -779,16 +779,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4444479999947362</v>
-      </c>
-      <c r="C2" t="n">
-        <v>17.00690800610012</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.00943873668482</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.82273619608103</v>
+        <v>92.05952316697221</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.26016468369701</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.43617303478057</v>
+      </c>
+      <c r="E2" t="n">
+        <v>28.33692434273317</v>
       </c>
     </row>
   </sheetData>
@@ -837,16 +837,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.465946625045035</v>
-      </c>
-      <c r="C2" t="n">
-        <v>31.00813685680638</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.89034747128728</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.92497855028857</v>
+        <v>96.39900233305525</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.88607447242882</v>
+      </c>
+      <c r="D2" t="n">
+        <v>39.03785127701862</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.34396934834961</v>
       </c>
     </row>
   </sheetData>
@@ -895,16 +895,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4868000840069726</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.64911993215144</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.13502423927772</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19.65145921281609</v>
+        <v>96.91558979201363</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.5585949920647</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.74642178704828</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40.23326735722674</v>
       </c>
     </row>
   </sheetData>
@@ -953,16 +953,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4979628750006668</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.50463608638653</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.27889223747904</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19.65057772937004</v>
+        <v>96.43836924998323</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.37538733786506</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.09874295284713</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.66499531550286</v>
       </c>
     </row>
   </sheetData>
@@ -1011,16 +1011,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4584064579685219</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.2121574722048</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.10603694028834</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.77401860556446</v>
+        <v>93.29169045900926</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.43674818938148</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.95806403129205</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.10981674646867</v>
       </c>
     </row>
   </sheetData>
@@ -1069,16 +1069,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4831453750375658</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.83183529816539</v>
-      </c>
-      <c r="D2" t="n">
-        <v>29.45710062424993</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.89905852237957</v>
+        <v>91.75059145898558</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.92435542868784</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.50254483991819</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.31447341565362</v>
       </c>
     </row>
   </sheetData>
@@ -1127,16 +1127,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.462198042019736</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.94998130234309</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.23575712932427</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.98515992723572</v>
+        <v>94.76651312503964</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.0760083773454</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.46787792057069</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.63452901797182</v>
       </c>
     </row>
   </sheetData>
@@ -1185,16 +1185,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4559938330203295</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.65454349197824</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.40994515248718</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18.6318910481627</v>
+        <v>93.50799925002502</v>
+      </c>
+      <c r="C2" t="n">
+        <v>41.47936574227342</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.7974285673054</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.40592064161327</v>
       </c>
     </row>
   </sheetData>
@@ -1243,16 +1243,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4895740420324728</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.79575761516885</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.95532388556797</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19.5070378448868</v>
+        <v>102.8696352500119</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.57157908740582</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.87566736591665</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.65962831502831</v>
       </c>
     </row>
   </sheetData>
@@ -1301,16 +1301,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4317401250009425</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.22293504715211</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.50882958460146</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.21003273488564</v>
+        <v>86.59418912499677</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.31884759205192</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.54100378998753</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.80442604023087</v>
       </c>
     </row>
   </sheetData>
@@ -1359,16 +1359,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4597630420466885</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.62343496909598</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.14542949380088</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.2741676475846</v>
+        <v>96.6431414160179</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.33308988786536</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46.90123339586296</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.04621692962725</v>
       </c>
     </row>
   </sheetData>
@@ -1417,16 +1417,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4670543330139481</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.59280628259724</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.4102166286444</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.73619111489217</v>
+        <v>98.22585583396722</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.28076790222543</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.37366891614369</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.91905557447793</v>
       </c>
     </row>
   </sheetData>
@@ -1475,16 +1475,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4660161250503734</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.76571172923181</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.62377219439282</v>
-      </c>
-      <c r="E2" t="n">
-        <v>27.98749803563798</v>
+        <v>95.95394179201685</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.73439476400991</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.57114045380887</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.43072755915247</v>
       </c>
     </row>
   </sheetData>
@@ -1533,16 +1533,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5381659170379862</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.00231313109435</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.15581898341194</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.03239409468427</v>
+        <v>92.79533966694726</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.55206788387243</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.36599208085217</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.38547359185092</v>
       </c>
     </row>
   </sheetData>
@@ -1591,16 +1591,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4959650419768877</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.55713749138069</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.26444350406449</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.68628430057309</v>
+        <v>99.34865891601657</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.97831831531856</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.24199579583797</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.58490657993019</v>
       </c>
     </row>
   </sheetData>
@@ -1649,16 +1649,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5016826249775477</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.87995186440714</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.19202528733592</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19.51881615769969</v>
+        <v>97.46191974997055</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.43327271573381</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.886844701407</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.04664759542176</v>
       </c>
     </row>
   </sheetData>
@@ -1707,16 +1707,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6234678749460727</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.56810797227596</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.65740442886784</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.18124894574606</v>
+        <v>93.83982362499228</v>
+      </c>
+      <c r="C2" t="n">
+        <v>46.97214567148534</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.46444712482853</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.39123358477094</v>
       </c>
     </row>
   </sheetData>
@@ -1765,16 +1765,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4810379580012523</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.83250822760334</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.09957782678512</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.45477220404261</v>
+        <v>92.17984070797684</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.3568724418037</v>
+      </c>
+      <c r="D2" t="n">
+        <v>39.69765781281721</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.0357763351851</v>
       </c>
     </row>
   </sheetData>
@@ -1823,16 +1823,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4997442080057226</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.70329853361846</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.4893983873449</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.95786305008847</v>
+        <v>99.10200729098869</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.92543120127674</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.4101898943383</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.13180510380786</v>
       </c>
     </row>
   </sheetData>
@@ -1881,16 +1881,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4885054159676656</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.11570384633027</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.72653245488466</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.91127042067783</v>
+        <v>102.455897708016</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.01459017836324</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.57438092651077</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.263262707523</v>
       </c>
     </row>
   </sheetData>
@@ -1939,16 +1939,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4906524170073681</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.24729134342927</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.5332504543073</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.65513790142735</v>
+        <v>96.50011783302762</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.29227993552242</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.47255636139118</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.35452954309305</v>
       </c>
     </row>
   </sheetData>
@@ -1997,16 +1997,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.519642458006274</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.34005025958981</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.75457370222402</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.98089804887476</v>
+        <v>99.61890129098902</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.06612012192357</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.15824223909304</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.3043399092136</v>
       </c>
     </row>
   </sheetData>
@@ -2055,16 +2055,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4480422499473207</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.89448486362354</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.74795498143215</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.75097669276287</v>
+        <v>89.86559633299476</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.64220111328607</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.31134858776552</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40.13061512618592</v>
       </c>
     </row>
   </sheetData>
@@ -2113,16 +2113,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5130996670341119</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.78003520387707</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.38116581069173</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.12402027351215</v>
+        <v>105.9016978750005</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.53167635617375</v>
+      </c>
+      <c r="D2" t="n">
+        <v>42.78060054440017</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.00134651978826</v>
       </c>
     </row>
   </sheetData>
@@ -2171,16 +2171,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4642240829998627</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.89839112995375</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.99711043934022</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.08301563731496</v>
+        <v>95.31601166602923</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.22263706396372</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.19364806989471</v>
+      </c>
+      <c r="E2" t="n">
+        <v>31.81346912815138</v>
       </c>
     </row>
   </sheetData>
@@ -2229,16 +2229,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4921503330115229</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.72285511651527</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.35346408406875</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.76105930938301</v>
+        <v>101.4191446249606</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.86467206806592</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.02067009707997</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.24147829639951</v>
       </c>
     </row>
   </sheetData>
@@ -2287,16 +2287,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4216712919878773</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.79077990584302</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.75339071977798</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.88136462877876</v>
+        <v>85.49283549998654</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.39348039565034</v>
+      </c>
+      <c r="D2" t="n">
+        <v>45.68199794514776</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.32367535976977</v>
       </c>
     </row>
   </sheetData>
@@ -2345,16 +2345,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4436407499597408</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.9120502981782</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.20680006472181</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.76842906184633</v>
+        <v>92.6374113750062</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.31709551384567</v>
+      </c>
+      <c r="D2" t="n">
+        <v>34.60036157724502</v>
+      </c>
+      <c r="E2" t="n">
+        <v>42.91674814252808</v>
       </c>
     </row>
   </sheetData>
@@ -2403,16 +2403,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4445610830443911</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.44175294888361</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.31986188292599</v>
-      </c>
-      <c r="E2" t="n">
-        <v>16.68787996953534</v>
+        <v>87.35151850001421</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.70181876850802</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.2573477481811</v>
+      </c>
+      <c r="E2" t="n">
+        <v>29.83129371271167</v>
       </c>
     </row>
   </sheetData>
@@ -2461,16 +2461,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4694024579948746</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.96184797777165</v>
-      </c>
-      <c r="D2" t="n">
-        <v>16.87450315692069</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.76230279894002</v>
+        <v>98.11960291699506</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.96627394943871</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.1715644357061</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.89734248338902</v>
       </c>
     </row>
   </sheetData>
@@ -2519,16 +2519,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4908002919983119</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.94666315233257</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.31926581905606</v>
-      </c>
-      <c r="E2" t="n">
-        <v>30.15147987451761</v>
+        <v>100.7348484579707</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.52146118433598</v>
+      </c>
+      <c r="D2" t="n">
+        <v>41.83262600837593</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.40139913123631</v>
       </c>
     </row>
   </sheetData>
@@ -2577,16 +2577,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4754954579984769</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.99010449704049</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.88297630502865</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.01427917512165</v>
+        <v>99.17766166600632</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.7872710731656</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.06272717298109</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.79726259355773</v>
       </c>
     </row>
   </sheetData>
@@ -2635,16 +2635,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5073761660023592</v>
-      </c>
-      <c r="C2" t="n">
-        <v>30.37462218087012</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.28073607903753</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.42536327024472</v>
+        <v>93.98351208301028</v>
+      </c>
+      <c r="C2" t="n">
+        <v>49.60801851585195</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.55154704785413</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.08851238824451</v>
       </c>
     </row>
   </sheetData>
@@ -2693,16 +2693,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5347422499908134</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.44535745595522</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.4720350635183</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.76080246185071</v>
+        <v>100.6083785410156</v>
+      </c>
+      <c r="C2" t="n">
+        <v>41.1866329801953</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.08758219029632</v>
+      </c>
+      <c r="E2" t="n">
+        <v>42.13237780576402</v>
       </c>
     </row>
   </sheetData>
@@ -2751,16 +2751,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4585560420528054</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.31467894976188</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.1859606815307</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18.77516246403232</v>
+        <v>90.29213670798345</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.79995379316415</v>
+      </c>
+      <c r="D2" t="n">
+        <v>44.13020480021252</v>
+      </c>
+      <c r="E2" t="n">
+        <v>28.00889783427481</v>
       </c>
     </row>
   </sheetData>
@@ -2809,16 +2809,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4709887499921024</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.33621498906155</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.0693071132916</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.3561421015806</v>
+        <v>92.90918850002345</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.8855286614932</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.14377140154127</v>
+      </c>
+      <c r="E2" t="n">
+        <v>33.71752348465955</v>
       </c>
     </row>
   </sheetData>
@@ -2867,16 +2867,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5005467089940794</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.74520101977825</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.14523551996249</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.61976992011225</v>
+        <v>100.4831862079445</v>
+      </c>
+      <c r="C2" t="n">
+        <v>50.03858697626888</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.89291840710445</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.33958922873936</v>
       </c>
     </row>
   </sheetData>
@@ -2925,16 +2925,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4845495409681462</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.18372436578463</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.88998818760986</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.75069518221195</v>
+        <v>96.61025441699894</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.1560036909033</v>
+      </c>
+      <c r="D2" t="n">
+        <v>42.53599918373288</v>
+      </c>
+      <c r="E2" t="n">
+        <v>29.7813657850855</v>
       </c>
     </row>
   </sheetData>
@@ -2983,16 +2983,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4366817079717293</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.05754631267668</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.9774286878463</v>
-      </c>
-      <c r="E2" t="n">
-        <v>27.41008115697912</v>
+        <v>83.86304387502605</v>
+      </c>
+      <c r="C2" t="n">
+        <v>29.19185746211983</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.7585853540091</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.57043823790783</v>
       </c>
     </row>
   </sheetData>
@@ -3041,16 +3041,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4635234579909593</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.88556613747199</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.28456413129654</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.53852221544837</v>
+        <v>93.60646737500792</v>
+      </c>
+      <c r="C2" t="n">
+        <v>32.11562911750823</v>
+      </c>
+      <c r="D2" t="n">
+        <v>41.70016954030636</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.31250317382044</v>
       </c>
     </row>
   </sheetData>
@@ -3099,16 +3099,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.535453749995213</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.63503500698992</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.63483100729074</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.66018174715394</v>
+        <v>98.63903262495296</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.0825057970051</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.22524536094973</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.23831492509514</v>
       </c>
     </row>
   </sheetData>
@@ -3157,16 +3157,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4647326249978505</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.03877852955052</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.65115996104501</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.67817576069298</v>
+        <v>96.82054166699527</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.78252991832904</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.31266031597961</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.90888647440021</v>
       </c>
     </row>
   </sheetData>
@@ -3215,16 +3215,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5062364169862121</v>
-      </c>
-      <c r="C2" t="n">
-        <v>17.08329784729039</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.73249152993497</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.20045622976233</v>
+        <v>97.19126904103905</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.06770890880552</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.48372608815544</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.76629144874066</v>
       </c>
     </row>
   </sheetData>
@@ -3273,16 +3273,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4906185840372927</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.42085282647388</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.0715081682245</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.28147260547521</v>
+        <v>94.75640875002136</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.31741507095338</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.96309027484059</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.49246802198576</v>
       </c>
     </row>
   </sheetData>
@@ -3331,16 +3331,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4744691660162061</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.18182830980099</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.50532873129873</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.21631125166116</v>
+        <v>94.31096229201648</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.81228933484059</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.23061941698736</v>
+      </c>
+      <c r="E2" t="n">
+        <v>32.50907844877852</v>
       </c>
     </row>
   </sheetData>
@@ -3389,16 +3389,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4665580409928225</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.21954814865343</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.67258247743871</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.3787240340063</v>
+        <v>86.18774887500331</v>
+      </c>
+      <c r="C2" t="n">
+        <v>31.76787591880618</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.6285533291213</v>
+      </c>
+      <c r="E2" t="n">
+        <v>42.05611324829599</v>
       </c>
     </row>
   </sheetData>
@@ -3447,16 +3447,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4475172500242479</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.48033862620944</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.8419412890844</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.07622774982643</v>
+        <v>87.17286012496334</v>
+      </c>
+      <c r="C2" t="n">
+        <v>29.4971905640525</v>
+      </c>
+      <c r="D2" t="n">
+        <v>41.14702217801898</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.79960060865601</v>
       </c>
     </row>
   </sheetData>
@@ -3505,16 +3505,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4684934160322882</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.77696356258333</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.44092553836023</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.65646009921698</v>
+        <v>103.6505736249965</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.79083587400763</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.84565671263843</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.55996031491073</v>
       </c>
     </row>
   </sheetData>
@@ -3563,16 +3563,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.591002875007689</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.5853960258773</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.45240441553269</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.57398302893958</v>
+        <v>127.3856716250302</v>
+      </c>
+      <c r="C2" t="n">
+        <v>31.09656042711485</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.75496133644545</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.07367913408468</v>
       </c>
     </row>
   </sheetData>
@@ -3621,16 +3621,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5110510840313509</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.19741616541534</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.8496875408641</v>
-      </c>
-      <c r="E2" t="n">
-        <v>30.75350226266974</v>
+        <v>129.9016613340355</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.25660085079539</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.81371721887037</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.07036861922283</v>
       </c>
     </row>
   </sheetData>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4706832499941811</v>
-      </c>
-      <c r="C2" t="n">
-        <v>29.82806583782114</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.706985141456</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.93532210005397</v>
+        <v>102.1650997090037</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.59820315669437</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.04115565031524</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.29595005165726</v>
       </c>
     </row>
   </sheetData>
@@ -3737,16 +3737,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4923371669719927</v>
-      </c>
-      <c r="C2" t="n">
-        <v>14.89138236370202</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.53110986969676</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.99029828519781</v>
+        <v>95.32156154199038</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.45923942911268</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.6833852032805</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.15139736170723</v>
       </c>
     </row>
   </sheetData>
@@ -3795,16 +3795,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4688266249722801</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.82267397084231</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.95050432718226</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.65215576786471</v>
+        <v>97.02146808401449</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.43628583276184</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.9216875832531</v>
+      </c>
+      <c r="E2" t="n">
+        <v>31.51754912389751</v>
       </c>
     </row>
   </sheetData>
@@ -3853,16 +3853,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4474553329637274</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.78590725625953</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.73903138030521</v>
-      </c>
-      <c r="E2" t="n">
-        <v>27.28705936726029</v>
+        <v>90.35881820798386</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.58766423513552</v>
+      </c>
+      <c r="D2" t="n">
+        <v>34.36496750552016</v>
+      </c>
+      <c r="E2" t="n">
+        <v>34.5772452253911</v>
       </c>
     </row>
   </sheetData>
@@ -3911,16 +3911,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.505992874968797</v>
-      </c>
-      <c r="C2" t="n">
-        <v>16.6867258673639</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.6285469281454</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.8456488090459</v>
+        <v>109.5592702499707</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.8780679737992</v>
+      </c>
+      <c r="D2" t="n">
+        <v>34.55510029999395</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.34920501827825</v>
       </c>
     </row>
   </sheetData>
@@ -3969,16 +3969,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4676067079999484</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.19810898637325</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.51709284741425</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.51888043654487</v>
+        <v>112.5881753339781</v>
+      </c>
+      <c r="C2" t="n">
+        <v>44.09516142550884</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.57982194973352</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.15430732976218</v>
       </c>
     </row>
   </sheetData>
@@ -4027,16 +4027,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5083179579814896</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.64047096497753</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.90221528591419</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.57621760309757</v>
+        <v>119.7391382080386</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.91958959552854</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.14557421398687</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40.30995048802264</v>
       </c>
     </row>
   </sheetData>
@@ -4085,16 +4085,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4764979159808718</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.66348672204866</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.99273557404579</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19.62399509225227</v>
+        <v>110.9915144160041</v>
+      </c>
+      <c r="C2" t="n">
+        <v>32.07265569896474</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.8684578178421</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.74722618891121</v>
       </c>
     </row>
   </sheetData>
@@ -4143,16 +4143,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4647951250080951</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.07463094821438</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.98900481718714</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.08000365335933</v>
+        <v>92.07518154103309</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.40266774112518</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.36684183202388</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.02489491097608</v>
       </c>
     </row>
   </sheetData>
@@ -4201,16 +4201,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5097295420127921</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.79762327731885</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.88055451122178</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.22149102388374</v>
+        <v>102.8759361249977</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.37228506919369</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.66039573300787</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.82875032016438</v>
       </c>
     </row>
   </sheetData>
@@ -4259,16 +4259,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5132584579987451</v>
-      </c>
-      <c r="C2" t="n">
-        <v>17.538424703042</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.29700373618786</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.28243400286106</v>
+        <v>105.5439621250262</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.18613502804843</v>
+      </c>
+      <c r="D2" t="n">
+        <v>39.10936671678619</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.05348999361716</v>
       </c>
     </row>
   </sheetData>
@@ -4317,16 +4317,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.46409412502544</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.11107905521287</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.80829163873104</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.37568697544616</v>
+        <v>98.15748516697204</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.37887092316326</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.06661933528972</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.1540560887785</v>
       </c>
     </row>
   </sheetData>
@@ -4375,16 +4375,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4557956669596024</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.16061545075478</v>
-      </c>
-      <c r="D2" t="n">
-        <v>25.77415587142569</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.28143191866746</v>
+        <v>94.142239333014</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.18291990362067</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.39909823679685</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.17172575741287</v>
       </c>
     </row>
   </sheetData>
@@ -4433,16 +4433,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.466369166970253</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.04466586589898</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.54140291627496</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18.53182504676689</v>
+        <v>95.30948258400895</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.759168512813</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.06336394651878</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.87998499996576</v>
       </c>
     </row>
   </sheetData>
@@ -4491,16 +4491,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4328464579884894</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.37697123208543</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.38713136283944</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.56026802886137</v>
+        <v>87.64187458297238</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.07770640763228</v>
+      </c>
+      <c r="D2" t="n">
+        <v>39.71441276592004</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.82999812171149</v>
       </c>
     </row>
   </sheetData>
@@ -4549,16 +4549,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4634958750102669</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.29432336852135</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.71315647246158</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.28965480847966</v>
+        <v>89.24140437500319</v>
+      </c>
+      <c r="C2" t="n">
+        <v>41.59721165030261</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.71515944252949</v>
+      </c>
+      <c r="E2" t="n">
+        <v>33.69868964755393</v>
       </c>
     </row>
   </sheetData>
@@ -4607,16 +4607,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.448442833032459</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.71794047285356</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.72620290169245</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.5958891849228</v>
+        <v>90.52474483300466</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.9327796264406</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.41827647638502</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.26671254849914</v>
       </c>
     </row>
   </sheetData>
@@ -4665,16 +4665,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4507297499803826</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.84648976848758</v>
-      </c>
-      <c r="D2" t="n">
-        <v>26.14968882842515</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.91928228050764</v>
+        <v>86.74249212496215</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.02541196386321</v>
+      </c>
+      <c r="D2" t="n">
+        <v>41.41286544736148</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40.49939385684002</v>
       </c>
     </row>
   </sheetData>
@@ -4723,16 +4723,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4524475419893861</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.2521655695227</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.49465117963864</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.84941094930954</v>
+        <v>90.18214204203105</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.5958173186854</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.51757736101645</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.78426323232733</v>
       </c>
     </row>
   </sheetData>
@@ -4781,16 +4781,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4916767500108108</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.78687195323236</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.6193745074872</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.02731452409146</v>
+        <v>100.1356306250091</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.0027975697609</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.41489456299081</v>
+      </c>
+      <c r="E2" t="n">
+        <v>32.21853102880964</v>
       </c>
     </row>
   </sheetData>
@@ -4839,16 +4839,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4515878329984844</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.08733788948767</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.84551900028184</v>
-      </c>
-      <c r="E2" t="n">
-        <v>28.11910056807262</v>
+        <v>93.352932083013</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.54010765543507</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.38264971256394</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.37855671639612</v>
       </c>
     </row>
   </sheetData>
@@ -4897,16 +4897,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4522227080306038</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.84735217254053</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.61342991612037</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.23315232290549</v>
+        <v>89.15443258296</v>
+      </c>
+      <c r="C2" t="n">
+        <v>32.11904289576687</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.59021637481626</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.74779507922041</v>
       </c>
     </row>
   </sheetData>
@@ -4955,16 +4955,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4354380409931764</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.7290170740859</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.72101267545037</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.38361538021664</v>
+        <v>87.63462470803643</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.71814731370694</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.95535800884225</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.00617306521662</v>
       </c>
     </row>
   </sheetData>
@@ -5013,16 +5013,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4896254590130411</v>
-      </c>
-      <c r="C2" t="n">
-        <v>18.12702788940353</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.54008611986074</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.6068954530363</v>
+        <v>99.99132837500656</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.31722902987293</v>
+      </c>
+      <c r="D2" t="n">
+        <v>34.6918531058343</v>
+      </c>
+      <c r="E2" t="n">
+        <v>45.00721490764995</v>
       </c>
     </row>
   </sheetData>
@@ -5071,16 +5071,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4369553749565966</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.97084061679001</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.71253533154676</v>
-      </c>
-      <c r="E2" t="n">
-        <v>27.03617253979491</v>
+        <v>90.51657837501261</v>
+      </c>
+      <c r="C2" t="n">
+        <v>43.53072991581183</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.16977415021285</v>
+      </c>
+      <c r="E2" t="n">
+        <v>42.93807667807868</v>
       </c>
     </row>
   </sheetData>
@@ -5129,16 +5129,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.468365749984514</v>
-      </c>
-      <c r="C2" t="n">
-        <v>28.34648309698147</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.65151902447238</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.12546899366277</v>
+        <v>92.3811945830239</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.55477597719397</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31.28130898476313</v>
+      </c>
+      <c r="E2" t="n">
+        <v>37.03811833490424</v>
       </c>
     </row>
   </sheetData>
@@ -5187,16 +5187,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4692923750262707</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.34486495286399</v>
-      </c>
-      <c r="D2" t="n">
-        <v>27.35969790283003</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.46398124124504</v>
+        <v>96.37573920801515</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.48718555404724</v>
+      </c>
+      <c r="D2" t="n">
+        <v>44.94745868634217</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.9064469795595</v>
       </c>
     </row>
   </sheetData>
@@ -5245,16 +5245,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4772434160113335</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.83975753028188</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.25498691592523</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.97285421721046</v>
+        <v>93.86458537500584</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.68129772286658</v>
+      </c>
+      <c r="D2" t="n">
+        <v>34.73956153488641</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.21839953476471</v>
       </c>
     </row>
   </sheetData>
@@ -5303,16 +5303,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4919359580380842</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.58465009292101</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.6328603765918</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.00963681597158</v>
+        <v>93.93010341702029</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36.85049861013032</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.66053230291745</v>
+      </c>
+      <c r="E2" t="n">
+        <v>33.90435070286217</v>
       </c>
     </row>
   </sheetData>
@@ -5361,16 +5361,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4917407080065459</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.98759960016723</v>
-      </c>
-      <c r="D2" t="n">
-        <v>24.24768052131905</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.39352115195815</v>
+        <v>99.04172858298989</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.64314680724256</v>
+      </c>
+      <c r="D2" t="n">
+        <v>43.63718255129966</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40.64888165582985</v>
       </c>
     </row>
   </sheetData>
@@ -5419,16 +5419,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4913476249785163</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.20197042616092</v>
-      </c>
-      <c r="D2" t="n">
-        <v>16.23428468499328</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.63598278671747</v>
+        <v>97.2232100830297</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.88154859568248</v>
+      </c>
+      <c r="D2" t="n">
+        <v>29.18110814873896</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.61146735665387</v>
       </c>
     </row>
   </sheetData>
@@ -5477,16 +5477,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4673216249793768</v>
-      </c>
-      <c r="C2" t="n">
-        <v>26.27201012751401</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.43652452750934</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.81165256009826</v>
+        <v>95.1953547919984</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.09532231033349</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.16672794101622</v>
+      </c>
+      <c r="E2" t="n">
+        <v>32.43701249809545</v>
       </c>
     </row>
   </sheetData>
@@ -5535,16 +5535,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.44541558297351</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.82066493926655</v>
-      </c>
-      <c r="D2" t="n">
-        <v>18.39922247682232</v>
-      </c>
-      <c r="E2" t="n">
-        <v>26.96289504030613</v>
+        <v>85.30433616600931</v>
+      </c>
+      <c r="C2" t="n">
+        <v>40.84226175881417</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.68319562882173</v>
+      </c>
+      <c r="E2" t="n">
+        <v>32.27319222931792</v>
       </c>
     </row>
   </sheetData>
@@ -5593,16 +5593,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5546211249893531</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.21852060070938</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.60766482972788</v>
-      </c>
-      <c r="E2" t="n">
-        <v>20.49734773342902</v>
+        <v>87.59029416594421</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30.11235869383962</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.5821118293009</v>
+      </c>
+      <c r="E2" t="n">
+        <v>34.31600220443118</v>
       </c>
     </row>
   </sheetData>
@@ -5651,16 +5651,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5500937500037253</v>
-      </c>
-      <c r="C2" t="n">
-        <v>24.78762077525591</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.62000094243704</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.7284972954679</v>
+        <v>93.79541191697353</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.31298508973872</v>
+      </c>
+      <c r="D2" t="n">
+        <v>36.77773943848968</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.74901227615186</v>
       </c>
     </row>
   </sheetData>
@@ -5709,16 +5709,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4717242079786956</v>
-      </c>
-      <c r="C2" t="n">
-        <v>27.54411227459675</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.50353067995027</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.0153879874682</v>
+        <v>100.9920562920161</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45.72933295938833</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.75217808902099</v>
+      </c>
+      <c r="E2" t="n">
+        <v>43.30860144847468</v>
       </c>
     </row>
   </sheetData>
@@ -5767,16 +5767,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4936683340347372</v>
-      </c>
-      <c r="C2" t="n">
-        <v>22.08174210246872</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.74234653108165</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.04528804103016</v>
+        <v>99.45987858297303</v>
+      </c>
+      <c r="C2" t="n">
+        <v>37.42023834248624</v>
+      </c>
+      <c r="D2" t="n">
+        <v>46.70466401307051</v>
+      </c>
+      <c r="E2" t="n">
+        <v>36.06957434892423</v>
       </c>
     </row>
   </sheetData>
@@ -5825,16 +5825,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4451020419946872</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.20668360623221</v>
-      </c>
-      <c r="D2" t="n">
-        <v>19.37819904433649</v>
-      </c>
-      <c r="E2" t="n">
-        <v>22.44325352621723</v>
+        <v>91.6177449169918</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.28281620491641</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30.98978675613301</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.8073027003602</v>
       </c>
     </row>
   </sheetData>
@@ -5883,16 +5883,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.450111249985639</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.28964221302525</v>
-      </c>
-      <c r="D2" t="n">
-        <v>28.87038417907146</v>
-      </c>
-      <c r="E2" t="n">
-        <v>25.72328727125822</v>
+        <v>92.08650462504011</v>
+      </c>
+      <c r="C2" t="n">
+        <v>35.8559621813608</v>
+      </c>
+      <c r="D2" t="n">
+        <v>40.72847213841642</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.43804387613066</v>
       </c>
     </row>
   </sheetData>
@@ -5941,16 +5941,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4766037500230595</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.15918029270644</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.32861933153792</v>
-      </c>
-      <c r="E2" t="n">
-        <v>31.29804851166714</v>
+        <v>95.56915450002998</v>
+      </c>
+      <c r="C2" t="n">
+        <v>41.81344894518618</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.3375449941378</v>
+      </c>
+      <c r="E2" t="n">
+        <v>45.78906937522235</v>
       </c>
     </row>
   </sheetData>
@@ -5999,16 +5999,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5158780830097385</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.28717170208409</v>
-      </c>
-      <c r="D2" t="n">
-        <v>16.9912862784152</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.94991391491155</v>
+        <v>102.6631943749962</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.3069207916676</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.62132798130573</v>
+      </c>
+      <c r="E2" t="n">
+        <v>41.7956221296352</v>
       </c>
     </row>
   </sheetData>
@@ -6057,16 +6057,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5299277079757303</v>
-      </c>
-      <c r="C2" t="n">
-        <v>25.06714305646604</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.81641111800294</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.85841463737171</v>
+        <v>89.86264050001046</v>
+      </c>
+      <c r="C2" t="n">
+        <v>39.71734916512253</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.63033971019402</v>
+      </c>
+      <c r="E2" t="n">
+        <v>33.76943109418783</v>
       </c>
     </row>
   </sheetData>
@@ -6115,16 +6115,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.523060625011567</v>
-      </c>
-      <c r="C2" t="n">
-        <v>20.84699041360835</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.28650845520313</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.54990691218736</v>
+        <v>98.51349149999442</v>
+      </c>
+      <c r="C2" t="n">
+        <v>38.99115370311148</v>
+      </c>
+      <c r="D2" t="n">
+        <v>37.73602201054414</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.94522721120775</v>
       </c>
     </row>
   </sheetData>
@@ -6173,16 +6173,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4503189169918187</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.3461361185242</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.30177077514224</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.56980538535515</v>
+        <v>90.72741854196647</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.51252414543788</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.06587105116888</v>
+      </c>
+      <c r="E2" t="n">
+        <v>38.81086830716981</v>
       </c>
     </row>
   </sheetData>
@@ -6231,16 +6231,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4613249590038322</v>
-      </c>
-      <c r="C2" t="n">
-        <v>23.08902739094227</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20.58561804605174</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.98931101646416</v>
+        <v>91.14369745797012</v>
+      </c>
+      <c r="C2" t="n">
+        <v>42.90814726764804</v>
+      </c>
+      <c r="D2" t="n">
+        <v>35.58756196270602</v>
+      </c>
+      <c r="E2" t="n">
+        <v>39.08127937258739</v>
       </c>
     </row>
   </sheetData>
@@ -6289,16 +6289,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4654627499985509</v>
-      </c>
-      <c r="C2" t="n">
-        <v>21.11747382075638</v>
-      </c>
-      <c r="D2" t="n">
-        <v>21.50938134084864</v>
-      </c>
-      <c r="E2" t="n">
-        <v>21.60305376164397</v>
+        <v>93.9791562500177</v>
+      </c>
+      <c r="C2" t="n">
+        <v>33.46457242779274</v>
+      </c>
+      <c r="D2" t="n">
+        <v>32.35726626860679</v>
+      </c>
+      <c r="E2" t="n">
+        <v>44.94177084604436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>